<commit_message>
Refine D3 physical and persistent-rate contract
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_mapping_params.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_mapping_params.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
     <t>section</t>
   </si>
@@ -34,7 +34,7 @@
     <t>Q_value_soft</t>
   </si>
   <si>
-    <t>Q_rate</t>
+    <t>Q_persistent_rate</t>
   </si>
   <si>
     <t>aggregation</t>
@@ -64,10 +64,13 @@
     <t>lambda_base</t>
   </si>
   <si>
+    <t>legacy_aliases</t>
+  </si>
+  <si>
     <t>boundary_behavior</t>
   </si>
   <si>
-    <t>v2.2.0</t>
+    <t>v2.3.0</t>
   </si>
   <si>
     <t>True</t>
@@ -94,10 +97,13 @@
     <t>20.0</t>
   </si>
   <si>
-    <t>{'Q_value_hard': 0.5, 'Q_value_soft': 0.2, 'Q_rate': 0.3}</t>
+    <t>{'Q_value_hard': 0.5, 'Q_value_soft': 0.2, 'Q_persistent_rate': 0.3}</t>
   </si>
   <si>
     <t>0.75</t>
+  </si>
+  <si>
+    <t>{'Q_rate': 'Q_persistent_rate'}</t>
   </si>
   <si>
     <t>{'included_in_score': False, 'reason': 'Boundary occupancy overlaps D1 floor/freeze and D4 tail-distribution evidence.'}</t>
@@ -458,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -480,7 +486,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -491,7 +497,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -502,7 +508,7 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -513,7 +519,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -524,7 +530,7 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -535,7 +541,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -546,7 +552,7 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -557,7 +563,7 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -568,7 +574,7 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -579,7 +585,7 @@
         <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -590,7 +596,7 @@
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -601,7 +607,7 @@
         <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -612,7 +618,7 @@
         <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -623,7 +629,18 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine D3 boundary and persistent-rate contracts
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_mapping_params.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_mapping_params.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="43">
   <si>
     <t>section</t>
   </si>
@@ -58,19 +58,40 @@
     <t>k</t>
   </si>
   <si>
+    <t>soft_only</t>
+  </si>
+  <si>
+    <t>hard</t>
+  </si>
+  <si>
+    <t>component_weights</t>
+  </si>
+  <si>
+    <t>evidence_contract</t>
+  </si>
+  <si>
     <t>weights</t>
   </si>
   <si>
     <t>lambda_base</t>
   </si>
   <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>candidate_rebalance_sensitivity_only</t>
+  </si>
+  <si>
+    <t>candidate_reason_not_promoted</t>
+  </si>
+  <si>
     <t>legacy_aliases</t>
   </si>
   <si>
     <t>boundary_behavior</t>
   </si>
   <si>
-    <t>v2.3.0</t>
+    <t>v2.4.0</t>
   </si>
   <si>
     <t>True</t>
@@ -91,16 +112,31 @@
     <t>15.0</t>
   </si>
   <si>
-    <t>0.05</t>
-  </si>
-  <si>
-    <t>20.0</t>
+    <t>two_level_logistic</t>
+  </si>
+  <si>
+    <t>{'x0': 0.05, 'k': 20.0}</t>
+  </si>
+  <si>
+    <t>{'soft_only': 0.3, 'hard': 0.7}</t>
+  </si>
+  <si>
+    <t>mutually_exclusive_soft_only_episode_and_hard_persistent_core</t>
   </si>
   <si>
     <t>{'Q_value_hard': 0.5, 'Q_value_soft': 0.2, 'Q_persistent_rate': 0.3}</t>
   </si>
   <si>
     <t>0.75</t>
+  </si>
+  <si>
+    <t>frozen_v2.3_weights_with_v2.4_rate_construct_update</t>
+  </si>
+  <si>
+    <t>{'Q_value_hard': 0.45, 'Q_value_soft': 0.35, 'Q_persistent_rate': 0.2}</t>
+  </si>
+  <si>
+    <t>large_ORP3_soft-bound_reclassification_without_external_labels</t>
   </si>
   <si>
     <t>{'Q_rate': 'Q_persistent_rate'}</t>
@@ -464,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -486,7 +522,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -497,7 +533,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -508,7 +544,7 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -519,7 +555,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -530,7 +566,7 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -541,7 +577,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -552,7 +588,7 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -563,7 +599,7 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -574,7 +610,7 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -582,10 +618,10 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -593,54 +629,109 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
         <v>8</v>
       </c>
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" t="s">
-        <v>30</v>
+      <c r="B20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>